<commit_message>
Medição pavimento desportivo: acrescentar soleiras e calha de transição
Acrescenta, no fim da folha e com a mesma formatação, os artigos do MQT
ligados aos remates do pavimento desportivo:

- 3.9.1.6 Soleiras interiores 400 / 200 / 150 mm (14 / 34 / 14 ml, parcial)
- 3.9.1.8 Calha de aço inox - remates de transição (15 ml, provável)

As linhas anteriores não foram alteradas.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017ZLPAXCR4AKn4GrY9WZfER
</commit_message>
<xml_diff>
--- a/PAVIMENTO_DESPORTIVO_INTERIORES.xlsx
+++ b/PAVIMENTO_DESPORTIVO_INTERIORES.xlsx
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="110" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="133" uniqueCount="78">
   <si>
     <t>Folha de Medição Em Obra</t>
   </si>
@@ -265,6 +265,43 @@
   </si>
   <si>
     <t>Estores de rolo motorizados — Sala Gimnodesportivo</t>
+  </si>
+  <si>
+    <t>3.9.1.6</t>
+  </si>
+  <si>
+    <t>SOLEIRAS INT.
+Fornecimento e aplicação de Soleira em Betão Polimérico tipo Tubani ou equiv., a aplicar em vãos interiores e/ou como elemento de transição entre espaços, com uma epessura média de 30 a 50mm e cor a definir em obra.
+Incluí: Todos os trabalhos e materiais necessários para a execução de acordo com as indicações do fabricante, com os desenhos de pormenor, mapa de acabamentos e caderno de encargos.
+Deve ser verificado o desenho correspondente à secção de cada tramo de soleira em obra e/ou nos desenhos de pormenor do Projeto de Arquitetura.</t>
+  </si>
+  <si>
+    <t>3.9.1.6.1</t>
+  </si>
+  <si>
+    <t>Soleiras interiores — 400 mm de largura</t>
+  </si>
+  <si>
+    <t>PARCIAL</t>
+  </si>
+  <si>
+    <t>3.9.1.6.2</t>
+  </si>
+  <si>
+    <t>Soleiras interiores — 200 mm de largura</t>
+  </si>
+  <si>
+    <t>3.9.1.6.3</t>
+  </si>
+  <si>
+    <t>Soleiras interiores — 150 mm de largura</t>
+  </si>
+  <si>
+    <t>3.9.1.8</t>
+  </si>
+  <si>
+    <t>CALHA DE AÇO INOX - REMATES TRANSIÇÃO Fornecimento e aplicação de calha de aço inox para aplicar em remates de transição de pavimentos.
+Incluí: Todos os trabalhos e materiais necessários para a execução de acordo com as indicações do fabricante, com os desenhos de pormenor, mapa de acabamentos e caderno de encargos.</t>
   </si>
 </sst>
 </file>
@@ -1337,7 +1374,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D14AFBEF-1D54-4853-9843-18D6A01975AF}">
-  <dimension ref="A1:P84"/>
+  <dimension ref="A1:P94"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="67.33203125" customWidth="1"/>
@@ -2172,112 +2209,175 @@
       <c r="G54" s="16"/>
       <c r="H54" s="3"/>
     </row>
-    <row r="55" spans="1:16" s="8" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A55" s="25"/>
-      <c r="B55" s="26"/>
-      <c r="C55" s="48"/>
-      <c r="D55" s="48"/>
-      <c r="E55" s="56"/>
-      <c r="F55" s="48"/>
-      <c r="G55" s="27"/>
-    </row>
-    <row r="56" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A56" s="24"/>
-      <c r="B56" s="24"/>
-      <c r="C56" s="49"/>
-      <c r="D56" s="68"/>
-      <c r="E56" s="57"/>
-      <c r="F56" s="49"/>
-      <c r="G56" s="18"/>
-    </row>
-    <row r="57" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A57" s="18"/>
-      <c r="B57" s="18"/>
-      <c r="C57" s="46"/>
-      <c r="D57" s="69"/>
-      <c r="E57" s="58"/>
-      <c r="F57" s="46"/>
-      <c r="G57" s="18"/>
+    <row r="55" spans="1:16" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A55" s="17"/>
+      <c r="B55" s="17"/>
+      <c r="C55" s="55"/>
+      <c r="D55" s="67"/>
+      <c r="E55" s="55"/>
+      <c r="F55" s="55"/>
+      <c r="G55" s="18"/>
+      <c r="H55" s="3"/>
+    </row>
+    <row r="56" spans="1:16" ht="114.0" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A56" s="77" t="s">
+        <v>67</v>
+      </c>
+      <c r="B56" s="76" t="s">
+        <v>68</v>
+      </c>
+      <c r="C56" s="47"/>
+      <c r="D56" s="47"/>
+      <c r="E56" s="78" t="s">
+        <v>39</v>
+      </c>
+      <c r="F56" s="44"/>
+      <c r="G56" s="19"/>
+      <c r="H56" s="3"/>
+    </row>
+    <row r="57" spans="1:16" s="8" customFormat="1" ht="13.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A57" s="25"/>
+      <c r="B57" s="28"/>
+      <c r="C57" s="48"/>
+      <c r="D57" s="66"/>
+      <c r="E57" s="54"/>
+      <c r="F57" s="45"/>
+      <c r="G57" s="25"/>
+      <c r="H57" s="3"/>
     </row>
     <row r="58" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A58" s="18"/>
-      <c r="B58" s="18"/>
-      <c r="C58" s="46"/>
-      <c r="D58" s="69"/>
-      <c r="E58" s="58"/>
-      <c r="F58" s="46"/>
-      <c r="G58" s="18"/>
-    </row>
-    <row r="59" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A59" s="18"/>
-      <c r="B59" s="18"/>
-      <c r="C59" s="46"/>
-      <c r="D59" s="69"/>
-      <c r="E59" s="58"/>
-      <c r="F59" s="46"/>
+      <c r="A58" s="15" t="s">
+        <v>69</v>
+      </c>
+      <c r="B58" s="14" t="s">
+        <v>70</v>
+      </c>
+      <c r="C58" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D58" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E58" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="F58" s="38">
+        <v>14</v>
+      </c>
+      <c r="G58" s="16"/>
+      <c r="H58" s="3"/>
+    </row>
+    <row r="59" spans="1:16" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A59" s="15"/>
+      <c r="B59" s="14"/>
+      <c r="C59" s="14"/>
+      <c r="D59" s="21"/>
+      <c r="E59" s="23"/>
+      <c r="F59" s="36"/>
       <c r="G59" s="18"/>
+      <c r="H59" s="3"/>
     </row>
     <row r="60" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A60" s="18"/>
-      <c r="B60" s="18"/>
-      <c r="C60" s="46"/>
-      <c r="D60" s="69"/>
-      <c r="E60" s="58"/>
-      <c r="F60" s="46"/>
-      <c r="G60" s="18"/>
-    </row>
-    <row r="61" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A61" s="18"/>
-      <c r="B61" s="18"/>
-      <c r="C61" s="46"/>
-      <c r="D61" s="69"/>
-      <c r="E61" s="58"/>
-      <c r="F61" s="46"/>
+      <c r="A60" s="15" t="s">
+        <v>72</v>
+      </c>
+      <c r="B60" s="14" t="s">
+        <v>73</v>
+      </c>
+      <c r="C60" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D60" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E60" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="F60" s="38">
+        <v>34</v>
+      </c>
+      <c r="G60" s="16"/>
+      <c r="H60" s="3"/>
+    </row>
+    <row r="61" spans="1:16" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A61" s="15"/>
+      <c r="B61" s="14"/>
+      <c r="C61" s="14"/>
+      <c r="D61" s="21"/>
+      <c r="E61" s="23"/>
+      <c r="F61" s="36"/>
       <c r="G61" s="18"/>
+      <c r="H61" s="3"/>
     </row>
     <row r="62" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A62" s="18"/>
-      <c r="B62" s="18"/>
-      <c r="C62" s="46"/>
-      <c r="D62" s="69"/>
-      <c r="E62" s="58"/>
-      <c r="F62" s="46"/>
-      <c r="G62" s="18"/>
-    </row>
-    <row r="63" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A63" s="18"/>
-      <c r="B63" s="18"/>
-      <c r="C63" s="46"/>
-      <c r="D63" s="69"/>
-      <c r="E63" s="58"/>
-      <c r="F63" s="46"/>
+      <c r="A62" s="15" t="s">
+        <v>74</v>
+      </c>
+      <c r="B62" s="14" t="s">
+        <v>75</v>
+      </c>
+      <c r="C62" s="14" t="s">
+        <v>21</v>
+      </c>
+      <c r="D62" s="21" t="s">
+        <v>71</v>
+      </c>
+      <c r="E62" s="79" t="s">
+        <v>39</v>
+      </c>
+      <c r="F62" s="38">
+        <v>14</v>
+      </c>
+      <c r="G62" s="16"/>
+      <c r="H62" s="3"/>
+    </row>
+    <row r="63" spans="1:16" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A63" s="17"/>
+      <c r="B63" s="17"/>
+      <c r="C63" s="55"/>
+      <c r="D63" s="67"/>
+      <c r="E63" s="55"/>
+      <c r="F63" s="55"/>
       <c r="G63" s="18"/>
-    </row>
-    <row r="64" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A64" s="18"/>
-      <c r="B64" s="18"/>
-      <c r="C64" s="46"/>
-      <c r="D64" s="69"/>
-      <c r="E64" s="58"/>
-      <c r="F64" s="46"/>
-      <c r="G64" s="18"/>
-    </row>
-    <row r="65" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A65" s="18"/>
-      <c r="B65" s="18"/>
-      <c r="C65" s="46"/>
-      <c r="D65" s="69"/>
-      <c r="E65" s="58"/>
-      <c r="F65" s="46"/>
-      <c r="G65" s="18"/>
+      <c r="H63" s="3"/>
+    </row>
+    <row r="64" spans="1:16" ht="66.0" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A64" s="86" t="s">
+        <v>76</v>
+      </c>
+      <c r="B64" s="81" t="s">
+        <v>77</v>
+      </c>
+      <c r="C64" s="82" t="s">
+        <v>21</v>
+      </c>
+      <c r="D64" s="83" t="s">
+        <v>22</v>
+      </c>
+      <c r="E64" s="84" t="s">
+        <v>39</v>
+      </c>
+      <c r="F64" s="85">
+        <v>15</v>
+      </c>
+      <c r="G64" s="27"/>
+    </row>
+    <row r="65" spans="1:16" s="8" customFormat="1" ht="13.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A65" s="25"/>
+      <c r="B65" s="26"/>
+      <c r="C65" s="48"/>
+      <c r="D65" s="48"/>
+      <c r="E65" s="56"/>
+      <c r="F65" s="48"/>
+      <c r="G65" s="27"/>
     </row>
     <row r="66" spans="1:16" x14ac:dyDescent="0.3">
-      <c r="A66" s="18"/>
-      <c r="B66" s="18"/>
-      <c r="C66" s="46"/>
-      <c r="D66" s="69"/>
-      <c r="E66" s="58"/>
-      <c r="F66" s="46"/>
+      <c r="A66" s="24"/>
+      <c r="B66" s="24"/>
+      <c r="C66" s="49"/>
+      <c r="D66" s="68"/>
+      <c r="E66" s="57"/>
+      <c r="F66" s="49"/>
       <c r="G66" s="18"/>
     </row>
     <row r="67" spans="1:16" x14ac:dyDescent="0.3">
@@ -2441,6 +2541,96 @@
       <c r="E84" s="58"/>
       <c r="F84" s="46"/>
       <c r="G84" s="18"/>
+    </row>
+    <row r="85" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A85" s="18"/>
+      <c r="B85" s="18"/>
+      <c r="C85" s="46"/>
+      <c r="D85" s="69"/>
+      <c r="E85" s="58"/>
+      <c r="F85" s="46"/>
+      <c r="G85" s="18"/>
+    </row>
+    <row r="86" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A86" s="18"/>
+      <c r="B86" s="18"/>
+      <c r="C86" s="46"/>
+      <c r="D86" s="69"/>
+      <c r="E86" s="58"/>
+      <c r="F86" s="46"/>
+      <c r="G86" s="18"/>
+    </row>
+    <row r="87" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A87" s="18"/>
+      <c r="B87" s="18"/>
+      <c r="C87" s="46"/>
+      <c r="D87" s="69"/>
+      <c r="E87" s="58"/>
+      <c r="F87" s="46"/>
+      <c r="G87" s="18"/>
+    </row>
+    <row r="88" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A88" s="18"/>
+      <c r="B88" s="18"/>
+      <c r="C88" s="46"/>
+      <c r="D88" s="69"/>
+      <c r="E88" s="58"/>
+      <c r="F88" s="46"/>
+      <c r="G88" s="18"/>
+    </row>
+    <row r="89" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A89" s="18"/>
+      <c r="B89" s="18"/>
+      <c r="C89" s="46"/>
+      <c r="D89" s="69"/>
+      <c r="E89" s="58"/>
+      <c r="F89" s="46"/>
+      <c r="G89" s="18"/>
+    </row>
+    <row r="90" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A90" s="18"/>
+      <c r="B90" s="18"/>
+      <c r="C90" s="46"/>
+      <c r="D90" s="69"/>
+      <c r="E90" s="58"/>
+      <c r="F90" s="46"/>
+      <c r="G90" s="18"/>
+    </row>
+    <row r="91" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A91" s="18"/>
+      <c r="B91" s="18"/>
+      <c r="C91" s="46"/>
+      <c r="D91" s="69"/>
+      <c r="E91" s="58"/>
+      <c r="F91" s="46"/>
+      <c r="G91" s="18"/>
+    </row>
+    <row r="92" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A92" s="18"/>
+      <c r="B92" s="18"/>
+      <c r="C92" s="46"/>
+      <c r="D92" s="69"/>
+      <c r="E92" s="58"/>
+      <c r="F92" s="46"/>
+      <c r="G92" s="18"/>
+    </row>
+    <row r="93" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A93" s="18"/>
+      <c r="B93" s="18"/>
+      <c r="C93" s="46"/>
+      <c r="D93" s="69"/>
+      <c r="E93" s="58"/>
+      <c r="F93" s="46"/>
+      <c r="G93" s="18"/>
+    </row>
+    <row r="94" spans="1:16" x14ac:dyDescent="0.3">
+      <c r="A94" s="18"/>
+      <c r="B94" s="18"/>
+      <c r="C94" s="46"/>
+      <c r="D94" s="69"/>
+      <c r="E94" s="58"/>
+      <c r="F94" s="46"/>
+      <c r="G94" s="18"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2588,6 +2778,34 @@
       <formula>$E52="OMISSÃO"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="D58:D62">
+    <cfRule type="expression" dxfId="3" priority="45">
+      <formula>$E58="TOTAL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="46">
+      <formula>$E58="PROVÁVEL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="47">
+      <formula>$E58="PARCIAL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="48">
+      <formula>$E58="OMISSÃO"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="D64">
+    <cfRule type="expression" dxfId="3" priority="49">
+      <formula>$E64="TOTAL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="50">
+      <formula>$E64="PROVÁVEL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="1" priority="51">
+      <formula>$E64="PARCIAL"</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="0" priority="52">
+      <formula>$E64="OMISSÃO"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>